<commit_message>
Update menu items: add descriptions, adjust prices, and replace dishes
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7e71a7f51efef439/Business/tripple/Digi Menu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0507C9AC-CDE9-41D0-9E67-AAEDBF44CB95}"/>
+  <xr:revisionPtr revIDLastSave="182" documentId="13_ncr:1_{EACECD44-A870-47B5-A715-DC205F132F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4A1CBFF-31B3-4809-821B-BFCCFEF80F80}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{FD36F3A3-C0BD-4176-B664-92451A287DD8}"/>
+    <workbookView xWindow="11190" yWindow="0" windowWidth="11460" windowHeight="14410" xr2:uid="{FD36F3A3-C0BD-4176-B664-92451A287DD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Menu" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="87">
   <si>
     <t>Espresso</t>
   </si>
@@ -252,6 +252,51 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>Caramel Frappe</t>
+  </si>
+  <si>
+    <t>Hazelnut Frappe</t>
+  </si>
+  <si>
+    <t>Chicken Club Sandwich</t>
+  </si>
+  <si>
+    <t>Add-ons</t>
+  </si>
+  <si>
+    <t>Extra shot</t>
+  </si>
+  <si>
+    <t>Extra cheese</t>
+  </si>
+  <si>
+    <t>Plain Fries</t>
+  </si>
+  <si>
+    <t>Loaded Fries</t>
+  </si>
+  <si>
+    <t>Extra Sausages</t>
+  </si>
+  <si>
+    <t>Extra Bread</t>
+  </si>
+  <si>
+    <t>Creamy Fettuccine</t>
+  </si>
+  <si>
+    <t>Beefy Bliss Burger</t>
+  </si>
+  <si>
+    <t>Fat Chick Burger</t>
+  </si>
+  <si>
+    <t>Crunchy Ceasar Bowl</t>
+  </si>
+  <si>
+    <t>Bean Protein Bowl</t>
   </si>
 </sst>
 </file>
@@ -639,7 +684,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C49F82-9CEF-4AC2-BDF7-287561CD6482}">
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.7265625" bestFit="1" customWidth="1"/>
@@ -648,7 +693,7 @@
     <col min="4" max="4" width="15.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -662,7 +707,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>29</v>
       </c>
@@ -670,10 +715,14 @@
         <v>0</v>
       </c>
       <c r="D2">
+        <f>E2/1.15</f>
         <v>391.304347826087</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>29</v>
       </c>
@@ -681,10 +730,14 @@
         <v>1</v>
       </c>
       <c r="D3">
+        <f t="shared" ref="D3:D75" si="0">E3/1.15</f>
         <v>608.69565217391312</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E3">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>29</v>
       </c>
@@ -692,10 +745,14 @@
         <v>11</v>
       </c>
       <c r="D4">
+        <f t="shared" si="0"/>
         <v>434.78260869565219</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E4">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>29</v>
       </c>
@@ -703,10 +760,14 @@
         <v>2</v>
       </c>
       <c r="D5">
+        <f t="shared" si="0"/>
         <v>565.21739130434787</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E5">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>29</v>
       </c>
@@ -714,10 +775,14 @@
         <v>3</v>
       </c>
       <c r="D6">
+        <f t="shared" si="0"/>
         <v>565.21739130434787</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E6">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>29</v>
       </c>
@@ -725,10 +790,14 @@
         <v>4</v>
       </c>
       <c r="D7">
+        <f t="shared" si="0"/>
         <v>695.6521739130435</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E7">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -736,10 +805,14 @@
         <v>5</v>
       </c>
       <c r="D8">
+        <f t="shared" si="0"/>
         <v>608.69565217391312</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E8">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>29</v>
       </c>
@@ -747,10 +820,14 @@
         <v>6</v>
       </c>
       <c r="D9">
+        <f t="shared" si="0"/>
         <v>739.13043478260875</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E9">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
@@ -758,10 +835,14 @@
         <v>7</v>
       </c>
       <c r="D10">
+        <f t="shared" si="0"/>
         <v>695.6521739130435</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E10">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
@@ -769,10 +850,14 @@
         <v>8</v>
       </c>
       <c r="D11">
+        <f t="shared" si="0"/>
         <v>695.6521739130435</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E11">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
@@ -780,10 +865,14 @@
         <v>12</v>
       </c>
       <c r="D12">
+        <f t="shared" si="0"/>
         <v>434.78260869565219</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E12">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
@@ -791,10 +880,14 @@
         <v>13</v>
       </c>
       <c r="D13">
+        <f t="shared" si="0"/>
         <v>565.21739130434787</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E13">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
@@ -802,10 +895,14 @@
         <v>14</v>
       </c>
       <c r="D14">
+        <f t="shared" si="0"/>
         <v>782.60869565217399</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E14">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
@@ -813,10 +910,14 @@
         <v>15</v>
       </c>
       <c r="D15">
+        <f t="shared" si="0"/>
         <v>782.60869565217399</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E15">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -824,10 +925,14 @@
         <v>16</v>
       </c>
       <c r="D16">
+        <f t="shared" si="0"/>
         <v>782.60869565217399</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E16">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
@@ -835,10 +940,14 @@
         <v>18</v>
       </c>
       <c r="D17">
+        <f t="shared" si="0"/>
         <v>869.56521739130437</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E17">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>30</v>
       </c>
@@ -846,10 +955,14 @@
         <v>17</v>
       </c>
       <c r="D18">
+        <f t="shared" si="0"/>
         <v>695.6521739130435</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E18">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
@@ -857,10 +970,14 @@
         <v>46</v>
       </c>
       <c r="D19">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E19">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
@@ -868,10 +985,14 @@
         <v>47</v>
       </c>
       <c r="D20">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E20">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
@@ -879,10 +1000,14 @@
         <v>48</v>
       </c>
       <c r="D21">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E21">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -890,10 +1015,14 @@
         <v>49</v>
       </c>
       <c r="D22">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E22">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -901,10 +1030,14 @@
         <v>51</v>
       </c>
       <c r="D23">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E23">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>31</v>
       </c>
@@ -912,10 +1045,14 @@
         <v>52</v>
       </c>
       <c r="D24">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E24">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
@@ -923,10 +1060,14 @@
         <v>53</v>
       </c>
       <c r="D25">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E25">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>31</v>
       </c>
@@ -934,10 +1075,14 @@
         <v>19</v>
       </c>
       <c r="D26">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E26">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>31</v>
       </c>
@@ -945,10 +1090,14 @@
         <v>20</v>
       </c>
       <c r="D27">
+        <f t="shared" si="0"/>
         <v>1043.4782608695652</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E27">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>31</v>
       </c>
@@ -956,10 +1105,14 @@
         <v>21</v>
       </c>
       <c r="D28">
+        <f t="shared" si="0"/>
         <v>869.56521739130437</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E28">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>31</v>
       </c>
@@ -967,359 +1120,701 @@
         <v>27</v>
       </c>
       <c r="D29">
+        <f t="shared" si="0"/>
         <v>869.56521739130437</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E29">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="D30">
-        <v>782.60869565217399</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>869.56521739130437</v>
+      </c>
+      <c r="E30">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="D31">
-        <v>782.60869565217399</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>869.56521739130437</v>
+      </c>
+      <c r="E31">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D32">
+        <f t="shared" si="0"/>
         <v>782.60869565217399</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E32">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B33" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33">
+        <f t="shared" si="0"/>
+        <v>782.60869565217399</v>
+      </c>
+      <c r="E33">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34">
+        <f t="shared" si="0"/>
+        <v>782.60869565217399</v>
+      </c>
+      <c r="E34">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" t="s">
         <v>38</v>
       </c>
-      <c r="D33">
+      <c r="D35">
+        <f t="shared" si="0"/>
         <v>782.60869565217399</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B34" t="s">
-        <v>50</v>
-      </c>
-      <c r="D34">
-        <v>739.13043478260875</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B35" t="s">
-        <v>23</v>
-      </c>
-      <c r="D35">
-        <v>739.13043478260875</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E35">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="D36">
-        <v>652.17391304347836</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>739.13043478260875</v>
+      </c>
+      <c r="E36">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B37" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="D37">
-        <v>608.69565217391312</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>739.13043478260875</v>
+      </c>
+      <c r="E37">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D38">
-        <v>521.73913043478262</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>652.17391304347836</v>
+      </c>
+      <c r="E38">
+        <v>750.00000000000011</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B39" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="D39">
-        <v>521.73913043478262</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>608.69565217391312</v>
+      </c>
+      <c r="E39">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="D40">
+        <f t="shared" si="0"/>
         <v>521.73913043478262</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E40">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B41" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41">
+        <f t="shared" si="0"/>
+        <v>521.73913043478262</v>
+      </c>
+      <c r="E41">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B42" t="s">
+        <v>61</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="0"/>
+        <v>521.73913043478262</v>
+      </c>
+      <c r="E42">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B43" t="s">
         <v>22</v>
       </c>
-      <c r="D41">
+      <c r="D43">
+        <f t="shared" si="0"/>
         <v>521.73913043478262</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B42" t="s">
-        <v>33</v>
-      </c>
-      <c r="D42">
-        <v>826.08695652173924</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B43" t="s">
-        <v>34</v>
-      </c>
-      <c r="D43">
-        <v>826.08695652173924</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E43">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B44" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="D44">
+        <f t="shared" si="0"/>
         <v>826.08695652173924</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E44">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B45" t="s">
+        <v>34</v>
+      </c>
+      <c r="D45">
+        <f t="shared" si="0"/>
+        <v>826.08695652173924</v>
+      </c>
+      <c r="E45">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B46" t="s">
+        <v>54</v>
+      </c>
+      <c r="D46">
+        <f t="shared" si="0"/>
+        <v>826.08695652173924</v>
+      </c>
+      <c r="E46">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B47" t="s">
         <v>55</v>
       </c>
-      <c r="D45">
+      <c r="D47">
+        <f t="shared" si="0"/>
         <v>826.08695652173924</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B46" t="s">
-        <v>57</v>
-      </c>
-      <c r="D46">
-        <v>826.08695652173924</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B47" t="s">
-        <v>56</v>
-      </c>
-      <c r="D47">
-        <v>739.13043478260875</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E47">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B48" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D48">
-        <v>739.13043478260875</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>826.08695652173924</v>
+      </c>
+      <c r="E48">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B49" t="s">
+        <v>56</v>
+      </c>
+      <c r="D49">
+        <f t="shared" si="0"/>
+        <v>739.13043478260875</v>
+      </c>
+      <c r="E49">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50" t="s">
+        <v>58</v>
+      </c>
+      <c r="D50">
+        <f t="shared" si="0"/>
+        <v>739.13043478260875</v>
+      </c>
+      <c r="E50">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B51" t="s">
         <v>59</v>
       </c>
-      <c r="D49">
+      <c r="D51">
+        <f t="shared" si="0"/>
         <v>608.69565217391312</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B50" t="s">
-        <v>63</v>
-      </c>
-      <c r="D50">
-        <v>956.52173913043487</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B51" t="s">
-        <v>64</v>
-      </c>
-      <c r="D51">
-        <v>608.69565217391312</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E51">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D52">
-        <v>869.56521739130437</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>956.52173913043487</v>
+      </c>
+      <c r="E52">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D53">
-        <v>782.60869565217399</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>608.69565217391312</v>
+      </c>
+      <c r="E53">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B54" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D54">
-        <v>1086.9565217391305</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+        <f t="shared" si="0"/>
+        <v>869.56521739130437</v>
+      </c>
+      <c r="E54">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B55" t="s">
+        <v>74</v>
+      </c>
+      <c r="D55">
+        <f t="shared" si="0"/>
+        <v>782.60869565217399</v>
+      </c>
+      <c r="E55">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B56" t="s">
+        <v>66</v>
+      </c>
+      <c r="D56">
+        <f t="shared" si="0"/>
+        <v>869.56521739130437</v>
+      </c>
+      <c r="E56">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A57" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" t="s">
+        <v>67</v>
+      </c>
+      <c r="D57">
+        <f t="shared" si="0"/>
+        <v>1304.3478260869567</v>
+      </c>
+      <c r="E57">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B58" t="s">
         <v>68</v>
       </c>
-      <c r="D55">
-        <v>1304.3478260869567</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" s="1" t="s">
+      <c r="D58">
+        <f t="shared" si="0"/>
+        <v>1521.7391304347827</v>
+      </c>
+      <c r="E58">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B59" t="s">
+        <v>82</v>
+      </c>
+      <c r="D59">
+        <f t="shared" si="0"/>
+        <v>1217.3913043478262</v>
+      </c>
+      <c r="E59">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" t="s">
+        <v>83</v>
+      </c>
+      <c r="D60">
+        <f t="shared" si="0"/>
+        <v>956.52173913043487</v>
+      </c>
+      <c r="E60">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B61" t="s">
+        <v>84</v>
+      </c>
+      <c r="D61">
+        <f t="shared" si="0"/>
+        <v>782.60869565217399</v>
+      </c>
+      <c r="E61">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62" t="s">
+        <v>85</v>
+      </c>
+      <c r="D62">
+        <f t="shared" si="0"/>
+        <v>1043.4782608695652</v>
+      </c>
+      <c r="E62">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>86</v>
+      </c>
+      <c r="D63">
+        <f t="shared" si="0"/>
+        <v>1043.4782608695652</v>
+      </c>
+      <c r="E63">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A64" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B64" t="s">
+        <v>78</v>
+      </c>
+      <c r="D64">
+        <f t="shared" si="0"/>
+        <v>434.78260869565219</v>
+      </c>
+      <c r="E64">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A65" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B65" t="s">
+        <v>79</v>
+      </c>
+      <c r="D65">
+        <f t="shared" si="0"/>
+        <v>695.6521739130435</v>
+      </c>
+      <c r="E65">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A66" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B66" t="s">
         <v>69</v>
       </c>
-      <c r="D56">
-        <v>608.69565217391312</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" s="1" t="s">
+      <c r="D66">
+        <f t="shared" si="0"/>
+        <v>695.6521739130435</v>
+      </c>
+      <c r="E66">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B67" t="s">
         <v>42</v>
       </c>
-      <c r="D57">
-        <v>695.6521739130435</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" s="1" t="s">
+      <c r="D67">
+        <f t="shared" si="0"/>
+        <v>869.56521739130437</v>
+      </c>
+      <c r="E67">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B68" t="s">
         <v>43</v>
       </c>
-      <c r="D58">
+      <c r="D68">
+        <f t="shared" si="0"/>
         <v>304.34782608695656</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" s="1" t="s">
+      <c r="E68">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B69" t="s">
         <v>44</v>
       </c>
-      <c r="D59">
+      <c r="D69">
+        <f t="shared" si="0"/>
         <v>347.82608695652175</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" s="1" t="s">
+      <c r="E69">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B70" t="s">
         <v>45</v>
       </c>
-      <c r="D60">
+      <c r="D70">
+        <f t="shared" si="0"/>
         <v>260.86956521739131</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" s="1" t="s">
+      <c r="E70">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B71" t="s">
         <v>70</v>
       </c>
-      <c r="D61">
+      <c r="D71">
+        <f t="shared" si="0"/>
         <v>260.86956521739131</v>
+      </c>
+      <c r="E71">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B72" t="s">
+        <v>76</v>
+      </c>
+      <c r="D72">
+        <f t="shared" si="0"/>
+        <v>217.39130434782609</v>
+      </c>
+      <c r="E72">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" t="s">
+        <v>77</v>
+      </c>
+      <c r="D73">
+        <f t="shared" si="0"/>
+        <v>173.91304347826087</v>
+      </c>
+      <c r="E73">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B74" t="s">
+        <v>80</v>
+      </c>
+      <c r="D74">
+        <f t="shared" si="0"/>
+        <v>217.39130434782609</v>
+      </c>
+      <c r="E74">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B75" t="s">
+        <v>81</v>
+      </c>
+      <c r="D75">
+        <f t="shared" si="0"/>
+        <v>86.956521739130437</v>
+      </c>
+      <c r="E75">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>